<commit_message>
Actualizo apadrinazgo: precios y plazos
</commit_message>
<xml_diff>
--- a/newsletter/newsletter_base_consolidada.xlsx
+++ b/newsletter/newsletter_base_consolidada.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uoe-my.sharepoint.com/personal/jzurita_ed_ac_uk/Documents/ArboretumMap/newsletter/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_E9AEEF77BF25873C1421F1BAF9147C3AA818AB73" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F7AF1031-ADBD-4834-ACFC-38922C4932EF}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="11_E9AEEF77BF25873C1421F1BAF9147C3AA818AB73" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2D53D5E0-2256-48B6-A94F-C9ED2A7E69B0}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="337">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="336">
   <si>
     <t>email</t>
   </si>
@@ -1040,9 +1040,6 @@
   </si>
   <si>
     <t>Caceres</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Golden </t>
   </si>
   <si>
     <t>Petrucci</t>
@@ -3380,7 +3377,9 @@
     <col min="1" max="1" width="35.7265625" style="8" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.1796875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.81640625" customWidth="1"/>
     <col min="5" max="5" width="10.7265625" customWidth="1"/>
+    <col min="7" max="7" width="11.453125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
@@ -3423,7 +3422,7 @@
         <v>2235951482</v>
       </c>
       <c r="F2" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
@@ -3440,7 +3439,7 @@
         <v>2235485135</v>
       </c>
       <c r="F3" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
@@ -3457,7 +3456,7 @@
         <v>2235418503</v>
       </c>
       <c r="F4" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
@@ -3471,7 +3470,7 @@
         <v>2235747922</v>
       </c>
       <c r="F5" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
@@ -3488,7 +3487,7 @@
         <v>2236980263</v>
       </c>
       <c r="F6" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
@@ -3496,16 +3495,16 @@
         <v>323</v>
       </c>
       <c r="B7" t="s">
+        <v>81</v>
+      </c>
+      <c r="C7" t="s">
         <v>332</v>
-      </c>
-      <c r="C7" t="s">
-        <v>333</v>
       </c>
       <c r="D7" s="9">
         <v>2235444704</v>
       </c>
       <c r="F7" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
@@ -3513,16 +3512,16 @@
         <v>324</v>
       </c>
       <c r="B8" t="s">
+        <v>333</v>
+      </c>
+      <c r="C8" t="s">
         <v>334</v>
-      </c>
-      <c r="C8" t="s">
-        <v>335</v>
       </c>
       <c r="D8" s="9">
         <v>2236337845</v>
       </c>
       <c r="F8" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
   </sheetData>

</xml_diff>